<commit_message>
feat: implement interactive dashboard with data visualizations and add demo video to documentation
</commit_message>
<xml_diff>
--- a/DOCS/burndown3.xlsx
+++ b/DOCS/burndown3.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="R:\FATEC\sem3\API-3\DOCS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D73798BD-D00E-433A-9B93-8DD1CC18EFEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB3701EE-7E53-4CCB-8243-DE35A2BE58ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Burn1" sheetId="1" r:id="rId1"/>
@@ -917,64 +917,64 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="21"/>
                 <c:pt idx="0">
-                  <c:v>28</c:v>
+                  <c:v>32</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>22</c:v>
+                  <c:v>26</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>17</c:v>
+                  <c:v>21</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>17</c:v>
+                  <c:v>21</c:v>
                 </c:pt>
                 <c:pt idx="4">
+                  <c:v>19</c:v>
+                </c:pt>
+                <c:pt idx="5">
                   <c:v>15</c:v>
                 </c:pt>
-                <c:pt idx="5">
-                  <c:v>11</c:v>
-                </c:pt>
                 <c:pt idx="6">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="8">
                   <c:v>8</c:v>
                 </c:pt>
-                <c:pt idx="7">
-                  <c:v>5</c:v>
-                </c:pt>
-                <c:pt idx="8">
+                <c:pt idx="9">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="10">
                   <c:v>4</c:v>
                 </c:pt>
-                <c:pt idx="9">
+                <c:pt idx="11">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="16">
                   <c:v>2</c:v>
                 </c:pt>
-                <c:pt idx="10">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="15">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="16">
-                  <c:v>0</c:v>
-                </c:pt>
                 <c:pt idx="17">
-                  <c:v>0</c:v>
+                  <c:v>2</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>0</c:v>
+                  <c:v>2</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>0</c:v>
+                  <c:v>2</c:v>
                 </c:pt>
                 <c:pt idx="20">
                   <c:v>0</c:v>
@@ -1091,64 +1091,64 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="21"/>
                 <c:pt idx="0">
-                  <c:v>28</c:v>
+                  <c:v>32</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>26.6</c:v>
+                  <c:v>30.4</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>25.2</c:v>
+                  <c:v>28.8</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>23.8</c:v>
+                  <c:v>27.2</c:v>
                 </c:pt>
                 <c:pt idx="4">
+                  <c:v>25.6</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>24</c:v>
+                </c:pt>
+                <c:pt idx="6">
                   <c:v>22.4</c:v>
                 </c:pt>
-                <c:pt idx="5">
-                  <c:v>21</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>19.600000000000001</c:v>
-                </c:pt>
                 <c:pt idx="7">
-                  <c:v>18.200000000000003</c:v>
+                  <c:v>20.799999999999997</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>16.8</c:v>
+                  <c:v>19.2</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>15.4</c:v>
+                  <c:v>17.600000000000001</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>14</c:v>
+                  <c:v>16</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>12.600000000000001</c:v>
+                  <c:v>14.399999999999999</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>11.200000000000003</c:v>
+                  <c:v>12.799999999999997</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>9.8000000000000007</c:v>
+                  <c:v>11.2</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>8.4000000000000021</c:v>
+                  <c:v>9.5999999999999979</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>7</c:v>
+                  <c:v>8</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>5.6000000000000014</c:v>
+                  <c:v>6.3999999999999986</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>4.2000000000000028</c:v>
+                  <c:v>4.7999999999999972</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>2.8000000000000007</c:v>
+                  <c:v>3.1999999999999993</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>1.4000000000000021</c:v>
+                  <c:v>1.5999999999999979</c:v>
                 </c:pt>
                 <c:pt idx="20">
                   <c:v>0</c:v>
@@ -1560,64 +1560,64 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="21"/>
                 <c:pt idx="0">
-                  <c:v>28</c:v>
+                  <c:v>32</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>22</c:v>
+                  <c:v>26</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>17</c:v>
+                  <c:v>21</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>17</c:v>
+                  <c:v>21</c:v>
                 </c:pt>
                 <c:pt idx="4">
+                  <c:v>19</c:v>
+                </c:pt>
+                <c:pt idx="5">
                   <c:v>15</c:v>
                 </c:pt>
-                <c:pt idx="5">
-                  <c:v>11</c:v>
-                </c:pt>
                 <c:pt idx="6">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="8">
                   <c:v>8</c:v>
                 </c:pt>
-                <c:pt idx="7">
-                  <c:v>5</c:v>
-                </c:pt>
-                <c:pt idx="8">
+                <c:pt idx="9">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="10">
                   <c:v>4</c:v>
                 </c:pt>
-                <c:pt idx="9">
+                <c:pt idx="11">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="16">
                   <c:v>2</c:v>
                 </c:pt>
-                <c:pt idx="10">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="15">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="16">
-                  <c:v>0</c:v>
-                </c:pt>
                 <c:pt idx="17">
-                  <c:v>0</c:v>
+                  <c:v>2</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>0</c:v>
+                  <c:v>2</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>0</c:v>
+                  <c:v>2</c:v>
                 </c:pt>
                 <c:pt idx="20">
                   <c:v>0</c:v>
@@ -1734,64 +1734,64 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="21"/>
                 <c:pt idx="0">
-                  <c:v>28</c:v>
+                  <c:v>32</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>26.6</c:v>
+                  <c:v>30.4</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>25.2</c:v>
+                  <c:v>28.8</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>23.8</c:v>
+                  <c:v>27.2</c:v>
                 </c:pt>
                 <c:pt idx="4">
+                  <c:v>25.6</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>24</c:v>
+                </c:pt>
+                <c:pt idx="6">
                   <c:v>22.4</c:v>
                 </c:pt>
-                <c:pt idx="5">
-                  <c:v>21</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>19.600000000000001</c:v>
-                </c:pt>
                 <c:pt idx="7">
-                  <c:v>18.200000000000003</c:v>
+                  <c:v>20.799999999999997</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>16.8</c:v>
+                  <c:v>19.2</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>15.4</c:v>
+                  <c:v>17.600000000000001</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>14</c:v>
+                  <c:v>16</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>12.600000000000001</c:v>
+                  <c:v>14.399999999999999</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>11.200000000000003</c:v>
+                  <c:v>12.799999999999997</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>9.8000000000000007</c:v>
+                  <c:v>11.2</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>8.4000000000000021</c:v>
+                  <c:v>9.5999999999999979</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>7</c:v>
+                  <c:v>8</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>5.6000000000000014</c:v>
+                  <c:v>6.3999999999999986</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>4.2000000000000028</c:v>
+                  <c:v>4.7999999999999972</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>2.8000000000000007</c:v>
+                  <c:v>3.1999999999999993</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>1.4000000000000021</c:v>
+                  <c:v>1.5999999999999979</c:v>
                 </c:pt>
                 <c:pt idx="20">
                   <c:v>0</c:v>
@@ -2628,7 +2628,7 @@
         <v>31</v>
       </c>
       <c r="B5" s="1">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="C5" s="1"/>
       <c r="D5" s="1"/>
@@ -2649,11 +2649,15 @@
       <c r="O5" s="1"/>
       <c r="P5" s="1"/>
       <c r="Q5" s="1"/>
-      <c r="R5" s="1"/>
+      <c r="R5" s="1">
+        <v>2</v>
+      </c>
       <c r="S5" s="1"/>
       <c r="T5" s="1"/>
       <c r="U5" s="1"/>
-      <c r="V5" s="1"/>
+      <c r="V5" s="1">
+        <v>2</v>
+      </c>
       <c r="W5" s="1">
         <f>Tabela2[[#This Row],[Total de horas]]-SUM(Tabela2[[#This Row],[Dia 1]:[Dia 20]])</f>
         <v>0</v>
@@ -2967,83 +2971,83 @@
       </c>
       <c r="B16" s="9">
         <f>SUM(B2:B15)</f>
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="C16" s="6">
         <f t="shared" ref="C16:V16" si="0">B16-SUM(C2:C15)</f>
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="D16" s="6">
         <f t="shared" si="0"/>
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="E16" s="6">
         <f t="shared" si="0"/>
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="F16" s="6">
         <f t="shared" si="0"/>
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="G16" s="6">
         <f t="shared" si="0"/>
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="H16" s="6">
         <f t="shared" si="0"/>
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="I16" s="9">
         <f t="shared" si="0"/>
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="J16" s="6">
         <f t="shared" si="0"/>
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="K16" s="6">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="L16" s="9">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="M16" s="6">
         <f>L16-SUM(M2:M15)</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="N16" s="6">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="O16" s="6">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="P16" s="6">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="Q16" s="6">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="R16" s="6">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="S16" s="6">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="T16" s="6">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="U16" s="6">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="V16" s="6">
         <f t="shared" si="0"/>
@@ -3057,83 +3061,83 @@
       </c>
       <c r="B17" s="8">
         <f>SUM(B2:B15)</f>
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="C17" s="7">
         <f t="shared" ref="C17:V17" si="1">$B$17-(($B$17/20)*(COLUMN()-2))</f>
-        <v>26.6</v>
+        <v>30.4</v>
       </c>
       <c r="D17" s="7">
         <f t="shared" si="1"/>
-        <v>25.2</v>
+        <v>28.8</v>
       </c>
       <c r="E17" s="7">
         <f t="shared" si="1"/>
-        <v>23.8</v>
+        <v>27.2</v>
       </c>
       <c r="F17" s="7">
         <f t="shared" si="1"/>
-        <v>22.4</v>
+        <v>25.6</v>
       </c>
       <c r="G17" s="7">
         <f t="shared" si="1"/>
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="H17" s="7">
         <f t="shared" si="1"/>
-        <v>19.600000000000001</v>
+        <v>22.4</v>
       </c>
       <c r="I17" s="7">
         <f t="shared" si="1"/>
-        <v>18.200000000000003</v>
+        <v>20.799999999999997</v>
       </c>
       <c r="J17" s="7">
         <f t="shared" si="1"/>
-        <v>16.8</v>
+        <v>19.2</v>
       </c>
       <c r="K17" s="7">
         <f t="shared" si="1"/>
-        <v>15.4</v>
+        <v>17.600000000000001</v>
       </c>
       <c r="L17" s="7">
         <f t="shared" si="1"/>
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="M17" s="7">
         <f t="shared" si="1"/>
-        <v>12.600000000000001</v>
+        <v>14.399999999999999</v>
       </c>
       <c r="N17" s="7">
         <f t="shared" si="1"/>
-        <v>11.200000000000003</v>
+        <v>12.799999999999997</v>
       </c>
       <c r="O17" s="7">
         <f t="shared" si="1"/>
-        <v>9.8000000000000007</v>
+        <v>11.2</v>
       </c>
       <c r="P17" s="7">
         <f t="shared" si="1"/>
-        <v>8.4000000000000021</v>
+        <v>9.5999999999999979</v>
       </c>
       <c r="Q17" s="7">
         <f t="shared" si="1"/>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="R17" s="7">
         <f t="shared" si="1"/>
-        <v>5.6000000000000014</v>
+        <v>6.3999999999999986</v>
       </c>
       <c r="S17" s="7">
         <f t="shared" si="1"/>
-        <v>4.2000000000000028</v>
+        <v>4.7999999999999972</v>
       </c>
       <c r="T17" s="7">
         <f t="shared" si="1"/>
-        <v>2.8000000000000007</v>
+        <v>3.1999999999999993</v>
       </c>
       <c r="U17" s="7">
         <f t="shared" si="1"/>
-        <v>1.4000000000000021</v>
+        <v>1.5999999999999979</v>
       </c>
       <c r="V17" s="7">
         <f t="shared" si="1"/>

</xml_diff>